<commit_message>
feat: app-wide responsiveness, notebook page number, and bulk import fixes
</commit_message>
<xml_diff>
--- a/public/assets/templates/customer_import_template.xlsx
+++ b/public/assets/templates/customer_import_template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="13">
   <si>
     <t>Name (Required)</t>
   </si>
@@ -51,6 +51,9 @@
   </si>
   <si>
     <t>Ali Motors</t>
+  </si>
+  <si>
+    <t>Page Number</t>
   </si>
 </sst>
 </file>
@@ -390,10 +393,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -415,8 +418,11 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
         <v>7</v>
       </c>

</xml_diff>